<commit_message>
cambios para recibir el excel
</commit_message>
<xml_diff>
--- a/data/format/DICCIONARIO DE DATOS - DM_188_METRICAS_GENERALES.xlsx
+++ b/data/format/DICCIONARIO DE DATOS - DM_188_METRICAS_GENERALES.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\kille\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{722AFAA6-0459-4A9D-B315-75115A4D69E9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{287FA33B-1446-4CAA-9652-9B36B16B7985}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="3" xr2:uid="{A31C2398-8C6B-42F8-8768-93FE8464293A}"/>
   </bookViews>
@@ -16,11 +16,11 @@
     <sheet name="Guía de Llenado" sheetId="4" r:id="rId1"/>
     <sheet name="Nivel Confidencialidad" sheetId="6" r:id="rId2"/>
     <sheet name="Clasificación de Datos Sensible" sheetId="5" r:id="rId3"/>
-    <sheet name="Mapeo de Campos" sheetId="1" r:id="rId4"/>
+    <sheet name="255568" sheetId="1" r:id="rId4"/>
     <sheet name="LISTAS" sheetId="3" state="hidden" r:id="rId5"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Mapeo de Campos'!$B$2:$K$10</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'255568'!$B$2:$K$10</definedName>
   </definedNames>
   <calcPr calcId="191028"/>
   <extLst>
@@ -277,7 +277,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="182" uniqueCount="121">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="242" uniqueCount="125">
   <si>
     <t>Diccionario de Datos</t>
   </si>
@@ -716,85 +716,97 @@
     <t>Text</t>
   </si>
   <si>
-    <t>id del registro/consulta</t>
-  </si>
-  <si>
-    <t>Id único de cada tienda. Concatenado entre MEGAPLAZA_CVE + TIENDA_CVE</t>
-  </si>
-  <si>
-    <t>Identificador único para realizar el JOIN de la tabla</t>
-  </si>
-  <si>
-    <t>fecha de consulta</t>
-  </si>
-  <si>
-    <t>Identificador de la Tabla</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Identificador del sistema fuente de información </t>
-  </si>
-  <si>
-    <t>Indica si es la última actualización para esa tabla periodo</t>
-  </si>
-  <si>
-    <t>Fecha que corresponde al periodo de la tabla</t>
-  </si>
-  <si>
-    <t>ID_CONSULTA</t>
-  </si>
-  <si>
-    <t>ID_TIENDA</t>
-  </si>
-  <si>
-    <t>CODIGO_TABLA</t>
-  </si>
-  <si>
-    <t>FECHA_CONSULTA</t>
-  </si>
-  <si>
-    <t>ID_TABLA</t>
-  </si>
-  <si>
-    <t>ID_FUENTE</t>
-  </si>
-  <si>
-    <t>ULTIMA_ACTUALIZACION</t>
-  </si>
-  <si>
-    <t>ID_PERIODO</t>
-  </si>
-  <si>
-    <t>VARCHAR</t>
-  </si>
-  <si>
-    <t>datetime</t>
-  </si>
-  <si>
-    <t>-</t>
-  </si>
-  <si>
-    <t>3</t>
-  </si>
-  <si>
-    <t>Abreviatura_Fuente + "_" + Abreviatura_Tabla + "_" + periodo + "_" +ID_Tienda + "_" + fecha_consulta("año""mes""dia", "hora", "minuto")</t>
-  </si>
-  <si>
-    <t>Calculada</t>
-  </si>
-  <si>
-    <t>Abreviatura_Tabla + periodo + "_" + TIENDA_ID</t>
-  </si>
-  <si>
-    <t>Año-Mes-Día-Hora-Minuto-Segundo</t>
-  </si>
-  <si>
-    <t>Abreviatura que corresponde a la tabla que se consultó</t>
-  </si>
-  <si>
-    <t>Alguno de los valores posibles.</t>
-  </si>
-  <si>
-    <t>Fecha asignada</t>
+    <t>TIENDA_KEY</t>
+  </si>
+  <si>
+    <t>SEMANA_ID</t>
+  </si>
+  <si>
+    <t>MES_ID</t>
+  </si>
+  <si>
+    <t>DIA_ID</t>
+  </si>
+  <si>
+    <t>CANTIDAD_REGISTROS</t>
+  </si>
+  <si>
+    <t>M1</t>
+  </si>
+  <si>
+    <t>M2</t>
+  </si>
+  <si>
+    <t>M3</t>
+  </si>
+  <si>
+    <t>M4</t>
+  </si>
+  <si>
+    <t>FECHA_MIN_CARGA</t>
+  </si>
+  <si>
+    <t>FECHA_MAX_CARGA</t>
+  </si>
+  <si>
+    <t>CONTEO_DIAS</t>
+  </si>
+  <si>
+    <t>CANTIDAD_BLANKS</t>
+  </si>
+  <si>
+    <t>CANTIDAD_COLUMNAS</t>
+  </si>
+  <si>
+    <t>SI</t>
+  </si>
+  <si>
+    <t>Identificador de la tienda</t>
+  </si>
+  <si>
+    <t>Identificador del periodo (solo para tablas semanales)</t>
+  </si>
+  <si>
+    <t>Identificador del periodo (solo para tablas mensuales)</t>
+  </si>
+  <si>
+    <t>Identificador del periodo (solo para tablas diarias)</t>
+  </si>
+  <si>
+    <t>Cantidad de registros para la tabla en ese periodo y para esa tienda en específico</t>
+  </si>
+  <si>
+    <t>Métrica 1: TOTAL_VENTA</t>
+  </si>
+  <si>
+    <t>Métrica 2: VENTA_PROMEDIO</t>
+  </si>
+  <si>
+    <t>Métrica 3: UNIDADES_VENDIDAS</t>
+  </si>
+  <si>
+    <t>Métrica 4: UNIDADES_VENDIDAS_PROMEDIO</t>
+  </si>
+  <si>
+    <t>Fecha mínima de carga</t>
+  </si>
+  <si>
+    <t>Fecha máxima de carga</t>
+  </si>
+  <si>
+    <t>Fecha máxima de carga - fecha mínima de carga</t>
+  </si>
+  <si>
+    <t>Cantidad de datos en blanco (en función de los campos obligatorios definidos)</t>
+  </si>
+  <si>
+    <t>Cantidad de columnas de la tabla.</t>
+  </si>
+  <si>
+    <t>Indefinido</t>
+  </si>
+  <si>
+    <t>N/A</t>
   </si>
 </sst>
 </file>
@@ -951,7 +963,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="30">
+  <borders count="33">
     <border>
       <left/>
       <right/>
@@ -1318,11 +1330,50 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="77">
+  <cellXfs count="78">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
@@ -1382,18 +1433,6 @@
     <xf numFmtId="0" fontId="11" fillId="6" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="23" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="24" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="25" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="26" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="9" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="justify" vertical="center" wrapText="1"/>
     </xf>
@@ -1549,6 +1588,19 @@
     </xf>
     <xf numFmtId="0" fontId="9" fillId="9" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="30" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="31" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="31" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="32" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -2223,336 +2275,336 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:12">
-      <c r="A1" s="52" t="e" vm="1">
+      <c r="A1" s="48" t="e" vm="1">
         <v>#VALUE!</v>
       </c>
-      <c r="B1" s="55" t="s">
+      <c r="B1" s="51" t="s">
         <v>0</v>
       </c>
-      <c r="C1" s="55"/>
-      <c r="D1" s="55"/>
-      <c r="E1" s="55"/>
-      <c r="F1" s="55"/>
-      <c r="G1" s="55"/>
-      <c r="H1" s="52"/>
-      <c r="I1" s="58"/>
+      <c r="C1" s="51"/>
+      <c r="D1" s="51"/>
+      <c r="E1" s="51"/>
+      <c r="F1" s="51"/>
+      <c r="G1" s="51"/>
+      <c r="H1" s="48"/>
+      <c r="I1" s="54"/>
     </row>
     <row r="2" spans="1:12">
-      <c r="A2" s="53"/>
-      <c r="B2" s="56"/>
-      <c r="C2" s="56"/>
-      <c r="D2" s="56"/>
-      <c r="E2" s="56"/>
-      <c r="F2" s="56"/>
-      <c r="G2" s="56"/>
-      <c r="H2" s="53"/>
-      <c r="I2" s="59"/>
+      <c r="A2" s="49"/>
+      <c r="B2" s="52"/>
+      <c r="C2" s="52"/>
+      <c r="D2" s="52"/>
+      <c r="E2" s="52"/>
+      <c r="F2" s="52"/>
+      <c r="G2" s="52"/>
+      <c r="H2" s="49"/>
+      <c r="I2" s="55"/>
     </row>
     <row r="3" spans="1:12" ht="15" thickBot="1">
-      <c r="A3" s="54"/>
-      <c r="B3" s="57"/>
-      <c r="C3" s="57"/>
-      <c r="D3" s="57"/>
-      <c r="E3" s="57"/>
-      <c r="F3" s="57"/>
-      <c r="G3" s="57"/>
-      <c r="H3" s="54"/>
-      <c r="I3" s="60"/>
+      <c r="A3" s="50"/>
+      <c r="B3" s="53"/>
+      <c r="C3" s="53"/>
+      <c r="D3" s="53"/>
+      <c r="E3" s="53"/>
+      <c r="F3" s="53"/>
+      <c r="G3" s="53"/>
+      <c r="H3" s="50"/>
+      <c r="I3" s="56"/>
     </row>
     <row r="4" spans="1:12" ht="9.6" customHeight="1" thickBot="1"/>
     <row r="5" spans="1:12">
-      <c r="A5" s="44" t="s">
+      <c r="A5" s="40" t="s">
         <v>1</v>
       </c>
-      <c r="B5" s="46" t="s">
+      <c r="B5" s="42" t="s">
         <v>2</v>
       </c>
-      <c r="C5" s="47"/>
-      <c r="D5" s="47"/>
-      <c r="E5" s="47"/>
-      <c r="F5" s="47"/>
-      <c r="G5" s="47"/>
-      <c r="H5" s="47"/>
-      <c r="I5" s="48"/>
+      <c r="C5" s="43"/>
+      <c r="D5" s="43"/>
+      <c r="E5" s="43"/>
+      <c r="F5" s="43"/>
+      <c r="G5" s="43"/>
+      <c r="H5" s="43"/>
+      <c r="I5" s="44"/>
     </row>
     <row r="6" spans="1:12" ht="15" thickBot="1">
-      <c r="A6" s="45"/>
-      <c r="B6" s="49"/>
-      <c r="C6" s="50"/>
-      <c r="D6" s="50"/>
-      <c r="E6" s="50"/>
-      <c r="F6" s="50"/>
-      <c r="G6" s="50"/>
-      <c r="H6" s="50"/>
-      <c r="I6" s="51"/>
+      <c r="A6" s="41"/>
+      <c r="B6" s="45"/>
+      <c r="C6" s="46"/>
+      <c r="D6" s="46"/>
+      <c r="E6" s="46"/>
+      <c r="F6" s="46"/>
+      <c r="G6" s="46"/>
+      <c r="H6" s="46"/>
+      <c r="I6" s="47"/>
     </row>
     <row r="7" spans="1:12" ht="8.5500000000000007" customHeight="1" thickBot="1">
-      <c r="A7" s="63"/>
-      <c r="B7" s="63"/>
-      <c r="C7" s="63"/>
-      <c r="D7" s="63"/>
-      <c r="E7" s="63"/>
-      <c r="F7" s="63"/>
-      <c r="G7" s="63"/>
-      <c r="H7" s="63"/>
-      <c r="I7" s="63"/>
+      <c r="A7" s="59"/>
+      <c r="B7" s="59"/>
+      <c r="C7" s="59"/>
+      <c r="D7" s="59"/>
+      <c r="E7" s="59"/>
+      <c r="F7" s="59"/>
+      <c r="G7" s="59"/>
+      <c r="H7" s="59"/>
+      <c r="I7" s="59"/>
     </row>
     <row r="8" spans="1:12" ht="15" thickBot="1"/>
     <row r="9" spans="1:12" ht="15" thickBot="1">
-      <c r="A9" s="64" t="s">
+      <c r="A9" s="60" t="s">
         <v>3</v>
       </c>
-      <c r="B9" s="65"/>
-      <c r="C9" s="65"/>
-      <c r="D9" s="65"/>
-      <c r="E9" s="65"/>
-      <c r="F9" s="65"/>
-      <c r="G9" s="65"/>
-      <c r="H9" s="65"/>
-      <c r="I9" s="66"/>
+      <c r="B9" s="61"/>
+      <c r="C9" s="61"/>
+      <c r="D9" s="61"/>
+      <c r="E9" s="61"/>
+      <c r="F9" s="61"/>
+      <c r="G9" s="61"/>
+      <c r="H9" s="61"/>
+      <c r="I9" s="62"/>
     </row>
     <row r="10" spans="1:12">
-      <c r="A10" s="28" t="s">
+      <c r="A10" s="24" t="s">
         <v>4</v>
       </c>
-      <c r="B10" s="67" t="s">
+      <c r="B10" s="63" t="s">
         <v>5</v>
       </c>
-      <c r="C10" s="67"/>
-      <c r="D10" s="67"/>
-      <c r="E10" s="67"/>
-      <c r="F10" s="67"/>
-      <c r="G10" s="67"/>
-      <c r="H10" s="67"/>
-      <c r="I10" s="68"/>
+      <c r="C10" s="63"/>
+      <c r="D10" s="63"/>
+      <c r="E10" s="63"/>
+      <c r="F10" s="63"/>
+      <c r="G10" s="63"/>
+      <c r="H10" s="63"/>
+      <c r="I10" s="64"/>
     </row>
     <row r="11" spans="1:12" ht="69" customHeight="1">
-      <c r="A11" s="29" t="s">
+      <c r="A11" s="25" t="s">
         <v>6</v>
       </c>
-      <c r="B11" s="40" t="s">
+      <c r="B11" s="36" t="s">
         <v>7</v>
       </c>
-      <c r="C11" s="40"/>
-      <c r="D11" s="40"/>
-      <c r="E11" s="40"/>
-      <c r="F11" s="40"/>
-      <c r="G11" s="40"/>
-      <c r="H11" s="40"/>
-      <c r="I11" s="41"/>
+      <c r="C11" s="36"/>
+      <c r="D11" s="36"/>
+      <c r="E11" s="36"/>
+      <c r="F11" s="36"/>
+      <c r="G11" s="36"/>
+      <c r="H11" s="36"/>
+      <c r="I11" s="37"/>
     </row>
     <row r="12" spans="1:12">
-      <c r="A12" s="29" t="s">
+      <c r="A12" s="25" t="s">
         <v>8</v>
       </c>
-      <c r="B12" s="61" t="s">
+      <c r="B12" s="57" t="s">
         <v>9</v>
       </c>
-      <c r="C12" s="61"/>
-      <c r="D12" s="61"/>
-      <c r="E12" s="61"/>
-      <c r="F12" s="61"/>
-      <c r="G12" s="61"/>
-      <c r="H12" s="61"/>
-      <c r="I12" s="62"/>
+      <c r="C12" s="57"/>
+      <c r="D12" s="57"/>
+      <c r="E12" s="57"/>
+      <c r="F12" s="57"/>
+      <c r="G12" s="57"/>
+      <c r="H12" s="57"/>
+      <c r="I12" s="58"/>
     </row>
     <row r="13" spans="1:12" ht="35.549999999999997" customHeight="1">
-      <c r="A13" s="29" t="s">
+      <c r="A13" s="25" t="s">
         <v>10</v>
       </c>
-      <c r="B13" s="40" t="s">
+      <c r="B13" s="36" t="s">
         <v>11</v>
       </c>
-      <c r="C13" s="40"/>
-      <c r="D13" s="40"/>
-      <c r="E13" s="40"/>
-      <c r="F13" s="40"/>
-      <c r="G13" s="40"/>
-      <c r="H13" s="40"/>
-      <c r="I13" s="41"/>
+      <c r="C13" s="36"/>
+      <c r="D13" s="36"/>
+      <c r="E13" s="36"/>
+      <c r="F13" s="36"/>
+      <c r="G13" s="36"/>
+      <c r="H13" s="36"/>
+      <c r="I13" s="37"/>
     </row>
     <row r="14" spans="1:12">
-      <c r="A14" s="29" t="s">
+      <c r="A14" s="25" t="s">
         <v>12</v>
       </c>
-      <c r="B14" s="61" t="s">
+      <c r="B14" s="57" t="s">
         <v>13</v>
       </c>
-      <c r="C14" s="61"/>
-      <c r="D14" s="61"/>
-      <c r="E14" s="61"/>
-      <c r="F14" s="61"/>
-      <c r="G14" s="61"/>
-      <c r="H14" s="61"/>
-      <c r="I14" s="62"/>
+      <c r="C14" s="57"/>
+      <c r="D14" s="57"/>
+      <c r="E14" s="57"/>
+      <c r="F14" s="57"/>
+      <c r="G14" s="57"/>
+      <c r="H14" s="57"/>
+      <c r="I14" s="58"/>
     </row>
     <row r="15" spans="1:12" ht="43.5" customHeight="1">
-      <c r="A15" s="29" t="s">
+      <c r="A15" s="25" t="s">
         <v>14</v>
       </c>
-      <c r="B15" s="40" t="s">
+      <c r="B15" s="36" t="s">
         <v>15</v>
       </c>
-      <c r="C15" s="40"/>
-      <c r="D15" s="40"/>
-      <c r="E15" s="40"/>
-      <c r="F15" s="40"/>
-      <c r="G15" s="40"/>
-      <c r="H15" s="40"/>
-      <c r="I15" s="41"/>
+      <c r="C15" s="36"/>
+      <c r="D15" s="36"/>
+      <c r="E15" s="36"/>
+      <c r="F15" s="36"/>
+      <c r="G15" s="36"/>
+      <c r="H15" s="36"/>
+      <c r="I15" s="37"/>
       <c r="J15" s="11"/>
       <c r="K15" s="11"/>
       <c r="L15" s="11"/>
     </row>
     <row r="16" spans="1:12" ht="82.05" customHeight="1">
-      <c r="A16" s="30" t="s">
+      <c r="A16" s="26" t="s">
         <v>16</v>
       </c>
-      <c r="B16" s="42" t="s">
+      <c r="B16" s="38" t="s">
         <v>17</v>
       </c>
-      <c r="C16" s="42"/>
-      <c r="D16" s="42"/>
-      <c r="E16" s="42"/>
-      <c r="F16" s="42"/>
-      <c r="G16" s="42"/>
-      <c r="H16" s="42"/>
-      <c r="I16" s="43"/>
+      <c r="C16" s="38"/>
+      <c r="D16" s="38"/>
+      <c r="E16" s="38"/>
+      <c r="F16" s="38"/>
+      <c r="G16" s="38"/>
+      <c r="H16" s="38"/>
+      <c r="I16" s="39"/>
     </row>
     <row r="17" spans="1:9">
-      <c r="A17" s="30" t="s">
+      <c r="A17" s="26" t="s">
         <v>18</v>
       </c>
-      <c r="B17" s="42" t="s">
+      <c r="B17" s="38" t="s">
         <v>19</v>
       </c>
-      <c r="C17" s="42"/>
-      <c r="D17" s="42"/>
-      <c r="E17" s="42"/>
-      <c r="F17" s="42"/>
-      <c r="G17" s="42"/>
-      <c r="H17" s="42"/>
-      <c r="I17" s="43"/>
+      <c r="C17" s="38"/>
+      <c r="D17" s="38"/>
+      <c r="E17" s="38"/>
+      <c r="F17" s="38"/>
+      <c r="G17" s="38"/>
+      <c r="H17" s="38"/>
+      <c r="I17" s="39"/>
     </row>
     <row r="18" spans="1:9">
-      <c r="A18" s="29" t="s">
+      <c r="A18" s="25" t="s">
         <v>20</v>
       </c>
-      <c r="B18" s="42" t="s">
+      <c r="B18" s="38" t="s">
         <v>21</v>
       </c>
-      <c r="C18" s="42"/>
-      <c r="D18" s="42"/>
-      <c r="E18" s="42"/>
-      <c r="F18" s="42"/>
-      <c r="G18" s="42"/>
-      <c r="H18" s="42"/>
-      <c r="I18" s="43"/>
+      <c r="C18" s="38"/>
+      <c r="D18" s="38"/>
+      <c r="E18" s="38"/>
+      <c r="F18" s="38"/>
+      <c r="G18" s="38"/>
+      <c r="H18" s="38"/>
+      <c r="I18" s="39"/>
     </row>
     <row r="19" spans="1:9">
-      <c r="A19" s="29" t="s">
+      <c r="A19" s="25" t="s">
         <v>22</v>
       </c>
-      <c r="B19" s="42" t="s">
+      <c r="B19" s="38" t="s">
         <v>23</v>
       </c>
-      <c r="C19" s="42"/>
-      <c r="D19" s="42"/>
-      <c r="E19" s="42"/>
-      <c r="F19" s="42"/>
-      <c r="G19" s="42"/>
-      <c r="H19" s="42"/>
-      <c r="I19" s="43"/>
+      <c r="C19" s="38"/>
+      <c r="D19" s="38"/>
+      <c r="E19" s="38"/>
+      <c r="F19" s="38"/>
+      <c r="G19" s="38"/>
+      <c r="H19" s="38"/>
+      <c r="I19" s="39"/>
     </row>
     <row r="20" spans="1:9">
-      <c r="A20" s="29" t="s">
+      <c r="A20" s="25" t="s">
         <v>24</v>
       </c>
-      <c r="B20" s="38" t="s">
+      <c r="B20" s="34" t="s">
         <v>25</v>
       </c>
-      <c r="C20" s="38"/>
-      <c r="D20" s="38"/>
-      <c r="E20" s="38"/>
-      <c r="F20" s="38"/>
-      <c r="G20" s="38"/>
-      <c r="H20" s="38"/>
-      <c r="I20" s="39"/>
+      <c r="C20" s="34"/>
+      <c r="D20" s="34"/>
+      <c r="E20" s="34"/>
+      <c r="F20" s="34"/>
+      <c r="G20" s="34"/>
+      <c r="H20" s="34"/>
+      <c r="I20" s="35"/>
     </row>
     <row r="21" spans="1:9" ht="14.55" customHeight="1">
-      <c r="A21" s="29" t="s">
+      <c r="A21" s="25" t="s">
         <v>26</v>
       </c>
-      <c r="B21" s="38" t="s">
+      <c r="B21" s="34" t="s">
         <v>27</v>
       </c>
-      <c r="C21" s="38"/>
-      <c r="D21" s="38"/>
-      <c r="E21" s="38"/>
-      <c r="F21" s="38"/>
-      <c r="G21" s="38"/>
-      <c r="H21" s="38"/>
-      <c r="I21" s="39"/>
+      <c r="C21" s="34"/>
+      <c r="D21" s="34"/>
+      <c r="E21" s="34"/>
+      <c r="F21" s="34"/>
+      <c r="G21" s="34"/>
+      <c r="H21" s="34"/>
+      <c r="I21" s="35"/>
     </row>
     <row r="22" spans="1:9" ht="14.55" customHeight="1">
-      <c r="A22" s="29" t="s">
+      <c r="A22" s="25" t="s">
         <v>28</v>
       </c>
-      <c r="B22" s="42" t="s">
+      <c r="B22" s="38" t="s">
         <v>29</v>
       </c>
-      <c r="C22" s="42"/>
-      <c r="D22" s="42"/>
-      <c r="E22" s="42"/>
-      <c r="F22" s="42"/>
-      <c r="G22" s="42"/>
-      <c r="H22" s="42"/>
-      <c r="I22" s="43"/>
+      <c r="C22" s="38"/>
+      <c r="D22" s="38"/>
+      <c r="E22" s="38"/>
+      <c r="F22" s="38"/>
+      <c r="G22" s="38"/>
+      <c r="H22" s="38"/>
+      <c r="I22" s="39"/>
     </row>
     <row r="23" spans="1:9" ht="14.55" customHeight="1">
-      <c r="A23" s="29" t="s">
+      <c r="A23" s="25" t="s">
         <v>30</v>
       </c>
-      <c r="B23" s="42" t="s">
+      <c r="B23" s="38" t="s">
         <v>31</v>
       </c>
-      <c r="C23" s="42"/>
-      <c r="D23" s="42"/>
-      <c r="E23" s="42"/>
-      <c r="F23" s="42"/>
-      <c r="G23" s="42"/>
-      <c r="H23" s="42"/>
-      <c r="I23" s="43"/>
+      <c r="C23" s="38"/>
+      <c r="D23" s="38"/>
+      <c r="E23" s="38"/>
+      <c r="F23" s="38"/>
+      <c r="G23" s="38"/>
+      <c r="H23" s="38"/>
+      <c r="I23" s="39"/>
     </row>
     <row r="24" spans="1:9" ht="14.55" customHeight="1">
-      <c r="A24" s="29" t="s">
+      <c r="A24" s="25" t="s">
         <v>32</v>
       </c>
-      <c r="B24" s="38" t="s">
+      <c r="B24" s="34" t="s">
         <v>33</v>
       </c>
-      <c r="C24" s="38"/>
-      <c r="D24" s="38"/>
-      <c r="E24" s="38"/>
-      <c r="F24" s="38"/>
-      <c r="G24" s="38"/>
-      <c r="H24" s="38"/>
-      <c r="I24" s="39"/>
+      <c r="C24" s="34"/>
+      <c r="D24" s="34"/>
+      <c r="E24" s="34"/>
+      <c r="F24" s="34"/>
+      <c r="G24" s="34"/>
+      <c r="H24" s="34"/>
+      <c r="I24" s="35"/>
     </row>
     <row r="25" spans="1:9" ht="31.5" customHeight="1" thickBot="1">
-      <c r="A25" s="31" t="s">
+      <c r="A25" s="27" t="s">
         <v>34</v>
       </c>
-      <c r="B25" s="36" t="s">
+      <c r="B25" s="32" t="s">
         <v>35</v>
       </c>
-      <c r="C25" s="36"/>
-      <c r="D25" s="36"/>
-      <c r="E25" s="36"/>
-      <c r="F25" s="36"/>
-      <c r="G25" s="36"/>
-      <c r="H25" s="36"/>
-      <c r="I25" s="37"/>
+      <c r="C25" s="32"/>
+      <c r="D25" s="32"/>
+      <c r="E25" s="32"/>
+      <c r="F25" s="32"/>
+      <c r="G25" s="32"/>
+      <c r="H25" s="32"/>
+      <c r="I25" s="33"/>
     </row>
   </sheetData>
   <mergeCells count="23">
@@ -2629,143 +2681,143 @@
       </c>
     </row>
     <row r="2" spans="1:3" ht="19.2">
-      <c r="A2" s="69" t="s">
+      <c r="A2" s="65" t="s">
         <v>39</v>
       </c>
-      <c r="B2" s="25" t="s">
+      <c r="B2" s="21" t="s">
         <v>40</v>
       </c>
-      <c r="C2" s="25" t="s">
+      <c r="C2" s="21" t="s">
         <v>41</v>
       </c>
     </row>
     <row r="3" spans="1:3" ht="19.2">
-      <c r="A3" s="70"/>
-      <c r="B3" s="25" t="s">
+      <c r="A3" s="66"/>
+      <c r="B3" s="21" t="s">
         <v>42</v>
       </c>
-      <c r="C3" s="25" t="s">
+      <c r="C3" s="21" t="s">
         <v>43</v>
       </c>
     </row>
     <row r="4" spans="1:3" ht="19.2">
-      <c r="A4" s="70"/>
-      <c r="B4" s="25" t="s">
+      <c r="A4" s="66"/>
+      <c r="B4" s="21" t="s">
         <v>44</v>
       </c>
-      <c r="C4" s="25" t="s">
+      <c r="C4" s="21" t="s">
         <v>45</v>
       </c>
     </row>
     <row r="5" spans="1:3" ht="28.8">
-      <c r="A5" s="70"/>
-      <c r="B5" s="25" t="s">
+      <c r="A5" s="66"/>
+      <c r="B5" s="21" t="s">
         <v>46</v>
       </c>
-      <c r="C5" s="25" t="s">
+      <c r="C5" s="21" t="s">
         <v>47</v>
       </c>
     </row>
     <row r="6" spans="1:3" ht="19.2">
-      <c r="A6" s="70"/>
-      <c r="B6" s="25" t="s">
+      <c r="A6" s="66"/>
+      <c r="B6" s="21" t="s">
         <v>48</v>
       </c>
-      <c r="C6" s="25" t="s">
+      <c r="C6" s="21" t="s">
         <v>49</v>
       </c>
     </row>
     <row r="7" spans="1:3" ht="19.2">
-      <c r="A7" s="70"/>
-      <c r="B7" s="25" t="s">
+      <c r="A7" s="66"/>
+      <c r="B7" s="21" t="s">
         <v>50</v>
       </c>
-      <c r="C7" s="25" t="s">
+      <c r="C7" s="21" t="s">
         <v>51</v>
       </c>
     </row>
     <row r="8" spans="1:3" ht="19.5" customHeight="1" thickBot="1">
-      <c r="A8" s="71"/>
-      <c r="B8" s="25" t="s">
+      <c r="A8" s="67"/>
+      <c r="B8" s="21" t="s">
         <v>52</v>
       </c>
-      <c r="C8" s="25" t="s">
+      <c r="C8" s="21" t="s">
         <v>53</v>
       </c>
     </row>
     <row r="9" spans="1:3" ht="38.4">
-      <c r="A9" s="72" t="s">
+      <c r="A9" s="68" t="s">
         <v>54</v>
       </c>
-      <c r="B9" s="26" t="s">
+      <c r="B9" s="22" t="s">
         <v>55</v>
       </c>
-      <c r="C9" s="26" t="s">
+      <c r="C9" s="22" t="s">
         <v>56</v>
       </c>
     </row>
     <row r="10" spans="1:3" ht="48">
-      <c r="A10" s="73"/>
-      <c r="B10" s="26" t="s">
+      <c r="A10" s="69"/>
+      <c r="B10" s="22" t="s">
         <v>57</v>
       </c>
-      <c r="C10" s="26" t="s">
+      <c r="C10" s="22" t="s">
         <v>58</v>
       </c>
     </row>
     <row r="11" spans="1:3" ht="28.8">
-      <c r="A11" s="73"/>
-      <c r="B11" s="26" t="s">
+      <c r="A11" s="69"/>
+      <c r="B11" s="22" t="s">
         <v>59</v>
       </c>
-      <c r="C11" s="26" t="s">
+      <c r="C11" s="22" t="s">
         <v>60</v>
       </c>
     </row>
     <row r="12" spans="1:3" ht="19.2">
-      <c r="A12" s="73"/>
-      <c r="B12" s="26" t="s">
+      <c r="A12" s="69"/>
+      <c r="B12" s="22" t="s">
         <v>61</v>
       </c>
-      <c r="C12" s="26" t="s">
+      <c r="C12" s="22" t="s">
         <v>62</v>
       </c>
     </row>
     <row r="13" spans="1:3" ht="19.2">
-      <c r="A13" s="73"/>
-      <c r="B13" s="26" t="s">
+      <c r="A13" s="69"/>
+      <c r="B13" s="22" t="s">
         <v>50</v>
       </c>
-      <c r="C13" s="26" t="s">
+      <c r="C13" s="22" t="s">
         <v>63</v>
       </c>
     </row>
     <row r="14" spans="1:3" ht="19.8" thickBot="1">
-      <c r="A14" s="74"/>
-      <c r="B14" s="26" t="s">
+      <c r="A14" s="70"/>
+      <c r="B14" s="22" t="s">
         <v>52</v>
       </c>
-      <c r="C14" s="26" t="s">
+      <c r="C14" s="22" t="s">
         <v>64</v>
       </c>
     </row>
     <row r="15" spans="1:3" ht="28.8">
-      <c r="A15" s="75" t="s">
+      <c r="A15" s="71" t="s">
         <v>65</v>
       </c>
-      <c r="B15" s="27" t="s">
+      <c r="B15" s="23" t="s">
         <v>66</v>
       </c>
-      <c r="C15" s="27" t="s">
+      <c r="C15" s="23" t="s">
         <v>67</v>
       </c>
     </row>
     <row r="16" spans="1:3" ht="19.8" thickBot="1">
-      <c r="A16" s="76"/>
-      <c r="B16" s="27" t="s">
+      <c r="A16" s="72"/>
+      <c r="B16" s="23" t="s">
         <v>68</v>
       </c>
-      <c r="C16" s="27" t="s">
+      <c r="C16" s="23" t="s">
         <v>69</v>
       </c>
     </row>
@@ -2785,10 +2837,10 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C02094D6-A0E8-4092-9184-0D999F8AEBED}">
-  <dimension ref="A1:N10"/>
+  <dimension ref="A1:N16"/>
   <sheetFormatPr defaultColWidth="11.33203125" defaultRowHeight="14.4"/>
   <cols>
-    <col min="1" max="1" width="13.5546875" style="34" customWidth="1"/>
+    <col min="1" max="1" width="13.5546875" style="30" customWidth="1"/>
     <col min="2" max="2" width="23.21875" style="7" customWidth="1"/>
     <col min="3" max="3" width="30.77734375" style="7" customWidth="1"/>
     <col min="4" max="4" width="26.33203125" bestFit="1" customWidth="1"/>
@@ -2799,25 +2851,25 @@
     <col min="9" max="9" width="23.77734375" style="7" customWidth="1"/>
     <col min="10" max="10" width="32.5546875" style="7" customWidth="1"/>
     <col min="11" max="11" width="36.33203125" style="7" customWidth="1"/>
-    <col min="12" max="14" width="10.77734375" style="33"/>
+    <col min="12" max="14" width="10.77734375" style="29"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:11" ht="51.6" customHeight="1" thickBot="1">
       <c r="A1" t="e" vm="1">
         <v>#VALUE!</v>
       </c>
-      <c r="B1" s="35" t="s">
+      <c r="B1" s="31" t="s">
         <v>70</v>
       </c>
-      <c r="C1" s="35"/>
-      <c r="D1" s="35"/>
-      <c r="E1" s="35"/>
-      <c r="F1" s="35"/>
-      <c r="G1" s="35"/>
-      <c r="H1" s="35"/>
-      <c r="I1" s="35"/>
-      <c r="J1" s="35"/>
-      <c r="K1" s="35"/>
+      <c r="C1" s="31"/>
+      <c r="D1" s="31"/>
+      <c r="E1" s="31"/>
+      <c r="F1" s="31"/>
+      <c r="G1" s="31"/>
+      <c r="H1" s="31"/>
+      <c r="I1" s="31"/>
+      <c r="J1" s="31"/>
+      <c r="K1" s="31"/>
     </row>
     <row r="2" spans="1:11" ht="16.2" thickBot="1">
       <c r="B2" s="12" t="s">
@@ -2852,244 +2904,434 @@
       </c>
     </row>
     <row r="3" spans="1:11" ht="15" thickBot="1">
-      <c r="B3" s="23" t="s">
-        <v>75</v>
-      </c>
-      <c r="C3" s="3" t="s">
-        <v>114</v>
-      </c>
-      <c r="D3" s="3" t="s">
-        <v>102</v>
-      </c>
-      <c r="E3" s="3" t="s">
+      <c r="B3" s="73" t="s">
+        <v>81</v>
+      </c>
+      <c r="C3" s="74" t="s">
+        <v>124</v>
+      </c>
+      <c r="D3" s="74" t="s">
         <v>94</v>
       </c>
-      <c r="F3" s="32">
-        <v>50</v>
+      <c r="E3" s="74" t="s">
+        <v>109</v>
+      </c>
+      <c r="F3" s="75" t="s">
+        <v>123</v>
       </c>
       <c r="G3" s="2" t="s">
-        <v>73</v>
+        <v>79</v>
       </c>
       <c r="H3" s="3" t="s">
+        <v>80</v>
+      </c>
+      <c r="I3" s="2" t="s">
+        <v>79</v>
+      </c>
+      <c r="J3" s="76" t="s">
+        <v>78</v>
+      </c>
+      <c r="K3" s="77" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="4" spans="1:11" ht="15" thickBot="1">
+      <c r="B4" s="73" t="s">
+        <v>81</v>
+      </c>
+      <c r="C4" s="74" t="s">
+        <v>124</v>
+      </c>
+      <c r="D4" s="3" t="s">
+        <v>95</v>
+      </c>
+      <c r="E4" s="3" t="s">
         <v>110</v>
       </c>
-      <c r="I3" s="32" t="s">
-        <v>79</v>
-      </c>
-      <c r="J3" s="6" t="s">
-        <v>78</v>
-      </c>
-      <c r="K3" s="22"/>
-    </row>
-    <row r="4" spans="1:11" ht="15" thickBot="1">
-      <c r="B4" s="23" t="s">
-        <v>75</v>
-      </c>
-      <c r="C4" s="3" t="s">
-        <v>115</v>
-      </c>
-      <c r="D4" s="3" t="s">
-        <v>103</v>
-      </c>
-      <c r="E4" s="3" t="s">
-        <v>95</v>
-      </c>
-      <c r="F4" s="32">
-        <v>10</v>
+      <c r="F4" s="28">
+        <v>6</v>
       </c>
       <c r="G4" s="2" t="s">
         <v>73</v>
       </c>
       <c r="H4" s="3" t="s">
-        <v>110</v>
-      </c>
-      <c r="I4" s="32" t="s">
-        <v>79</v>
-      </c>
-      <c r="J4" s="6" t="s">
+        <v>80</v>
+      </c>
+      <c r="I4" s="2" t="s">
+        <v>108</v>
+      </c>
+      <c r="J4" s="2" t="s">
         <v>78</v>
       </c>
-      <c r="K4" s="24"/>
+      <c r="K4" s="77" t="s">
+        <v>39</v>
+      </c>
     </row>
     <row r="5" spans="1:11" ht="15" thickBot="1">
-      <c r="B5" s="23" t="s">
-        <v>75</v>
-      </c>
-      <c r="C5" s="3" t="s">
-        <v>116</v>
+      <c r="B5" s="73" t="s">
+        <v>81</v>
+      </c>
+      <c r="C5" s="74" t="s">
+        <v>124</v>
       </c>
       <c r="D5" s="3" t="s">
-        <v>104</v>
+        <v>96</v>
       </c>
       <c r="E5" s="3" t="s">
-        <v>96</v>
-      </c>
-      <c r="F5" s="32">
-        <v>30</v>
-      </c>
-      <c r="G5" s="6" t="s">
+        <v>111</v>
+      </c>
+      <c r="F5" s="28">
+        <v>6</v>
+      </c>
+      <c r="G5" s="2" t="s">
         <v>73</v>
       </c>
       <c r="H5" s="3" t="s">
-        <v>110</v>
-      </c>
-      <c r="I5" s="32" t="s">
-        <v>79</v>
-      </c>
-      <c r="J5" s="6" t="s">
+        <v>80</v>
+      </c>
+      <c r="I5" s="2" t="s">
+        <v>108</v>
+      </c>
+      <c r="J5" s="2" t="s">
         <v>78</v>
       </c>
-      <c r="K5" s="24"/>
+      <c r="K5" s="77" t="s">
+        <v>39</v>
+      </c>
     </row>
     <row r="6" spans="1:11" ht="15" thickBot="1">
-      <c r="B6" s="21" t="s">
-        <v>75</v>
-      </c>
-      <c r="C6" s="3" t="s">
-        <v>117</v>
+      <c r="B6" s="73" t="s">
+        <v>81</v>
+      </c>
+      <c r="C6" s="74" t="s">
+        <v>124</v>
       </c>
       <c r="D6" s="3" t="s">
-        <v>105</v>
+        <v>97</v>
       </c>
       <c r="E6" s="3" t="s">
-        <v>97</v>
-      </c>
-      <c r="F6" s="3" t="s">
         <v>112</v>
+      </c>
+      <c r="F6" s="3">
+        <v>8</v>
       </c>
       <c r="G6" s="2" t="s">
         <v>73</v>
       </c>
       <c r="H6" s="3" t="s">
-        <v>111</v>
-      </c>
-      <c r="I6" s="32" t="s">
+        <v>80</v>
+      </c>
+      <c r="I6" s="2" t="s">
+        <v>108</v>
+      </c>
+      <c r="J6" s="2" t="s">
+        <v>78</v>
+      </c>
+      <c r="K6" s="77" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="7" spans="1:11" ht="15" thickBot="1">
+      <c r="B7" s="73" t="s">
+        <v>81</v>
+      </c>
+      <c r="C7" s="74" t="s">
+        <v>124</v>
+      </c>
+      <c r="D7" s="3" t="s">
+        <v>98</v>
+      </c>
+      <c r="E7" s="3" t="s">
+        <v>113</v>
+      </c>
+      <c r="F7" s="28"/>
+      <c r="G7" s="2" t="s">
         <v>79</v>
       </c>
-      <c r="J6" s="6" t="s">
+      <c r="H7" s="3" t="s">
+        <v>80</v>
+      </c>
+      <c r="I7" s="2" t="s">
+        <v>108</v>
+      </c>
+      <c r="J7" s="2" t="s">
         <v>78</v>
       </c>
-      <c r="K6" s="24"/>
-    </row>
-    <row r="7" spans="1:11" ht="15" thickBot="1">
-      <c r="B7" s="23" t="s">
-        <v>75</v>
-      </c>
-      <c r="C7" s="3" t="s">
-        <v>118</v>
-      </c>
-      <c r="D7" s="3" t="s">
-        <v>106</v>
-      </c>
-      <c r="E7" s="3" t="s">
-        <v>98</v>
-      </c>
-      <c r="F7" s="32">
-        <v>3</v>
-      </c>
-      <c r="G7" s="2" t="s">
-        <v>73</v>
-      </c>
-      <c r="H7" s="3" t="s">
-        <v>110</v>
-      </c>
-      <c r="I7" s="32" t="s">
+      <c r="K7" s="77" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="8" spans="1:11" ht="15" thickBot="1">
+      <c r="B8" s="73" t="s">
+        <v>81</v>
+      </c>
+      <c r="C8" s="74" t="s">
+        <v>124</v>
+      </c>
+      <c r="D8" s="3" t="s">
+        <v>99</v>
+      </c>
+      <c r="E8" s="3" t="s">
+        <v>114</v>
+      </c>
+      <c r="F8" s="28"/>
+      <c r="G8" s="2" t="s">
         <v>79</v>
       </c>
-      <c r="J7" s="6" t="s">
+      <c r="H8" s="3" t="s">
+        <v>80</v>
+      </c>
+      <c r="I8" s="2" t="s">
+        <v>108</v>
+      </c>
+      <c r="J8" s="2" t="s">
         <v>78</v>
       </c>
-      <c r="K7" s="24"/>
-    </row>
-    <row r="8" spans="1:11" ht="15" thickBot="1">
-      <c r="B8" s="23" t="s">
-        <v>75</v>
-      </c>
-      <c r="C8" s="3" t="s">
-        <v>119</v>
-      </c>
-      <c r="D8" s="3" t="s">
-        <v>107</v>
-      </c>
-      <c r="E8" s="3" t="s">
-        <v>99</v>
-      </c>
-      <c r="F8" s="32" t="s">
-        <v>113</v>
-      </c>
-      <c r="G8" s="2" t="s">
-        <v>73</v>
-      </c>
-      <c r="H8" s="3" t="s">
-        <v>110</v>
-      </c>
-      <c r="I8" s="32" t="s">
-        <v>79</v>
-      </c>
-      <c r="J8" s="6" t="s">
-        <v>78</v>
-      </c>
-      <c r="K8" s="24"/>
+      <c r="K8" s="77" t="s">
+        <v>39</v>
+      </c>
     </row>
     <row r="9" spans="1:11" ht="15" thickBot="1">
-      <c r="B9" s="23" t="s">
-        <v>75</v>
-      </c>
-      <c r="C9" s="3" t="s">
-        <v>119</v>
+      <c r="B9" s="73" t="s">
+        <v>81</v>
+      </c>
+      <c r="C9" s="74" t="s">
+        <v>124</v>
       </c>
       <c r="D9" s="3" t="s">
-        <v>108</v>
+        <v>100</v>
       </c>
       <c r="E9" s="3" t="s">
-        <v>100</v>
-      </c>
-      <c r="F9" s="3" t="s">
-        <v>112</v>
-      </c>
+        <v>115</v>
+      </c>
+      <c r="F9" s="3"/>
       <c r="G9" s="2" t="s">
         <v>79</v>
       </c>
       <c r="H9" s="3" t="s">
-        <v>89</v>
-      </c>
-      <c r="I9" s="32" t="s">
+        <v>80</v>
+      </c>
+      <c r="I9" s="2" t="s">
+        <v>108</v>
+      </c>
+      <c r="J9" s="2" t="s">
+        <v>78</v>
+      </c>
+      <c r="K9" s="77" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="10" spans="1:11" ht="15" thickBot="1">
+      <c r="B10" s="2" t="s">
+        <v>81</v>
+      </c>
+      <c r="C10" s="3" t="s">
+        <v>124</v>
+      </c>
+      <c r="D10" s="3" t="s">
+        <v>101</v>
+      </c>
+      <c r="E10" s="3" t="s">
+        <v>116</v>
+      </c>
+      <c r="F10" s="28"/>
+      <c r="G10" s="2" t="s">
         <v>79</v>
       </c>
-      <c r="J9" s="6" t="s">
+      <c r="H10" s="3" t="s">
+        <v>80</v>
+      </c>
+      <c r="I10" s="2" t="s">
+        <v>108</v>
+      </c>
+      <c r="J10" s="2" t="s">
         <v>78</v>
       </c>
-      <c r="K9" s="24"/>
-    </row>
-    <row r="10" spans="1:11">
-      <c r="B10" s="23" t="s">
-        <v>90</v>
-      </c>
-      <c r="C10" s="3" t="s">
+      <c r="K10" s="77" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="11" spans="1:11" ht="15" thickBot="1">
+      <c r="B11" s="2" t="s">
+        <v>81</v>
+      </c>
+      <c r="C11" s="3" t="s">
+        <v>124</v>
+      </c>
+      <c r="D11" s="3" t="s">
+        <v>102</v>
+      </c>
+      <c r="E11" s="3" t="s">
+        <v>117</v>
+      </c>
+      <c r="F11" s="3"/>
+      <c r="G11" s="2" t="s">
+        <v>79</v>
+      </c>
+      <c r="H11" s="3" t="s">
+        <v>80</v>
+      </c>
+      <c r="I11" s="2" t="s">
+        <v>108</v>
+      </c>
+      <c r="J11" s="2" t="s">
+        <v>78</v>
+      </c>
+      <c r="K11" s="77" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="12" spans="1:11" ht="15" thickBot="1">
+      <c r="B12" s="2" t="s">
+        <v>81</v>
+      </c>
+      <c r="C12" s="3" t="s">
+        <v>124</v>
+      </c>
+      <c r="D12" s="3" t="s">
+        <v>103</v>
+      </c>
+      <c r="E12" s="3" t="s">
+        <v>118</v>
+      </c>
+      <c r="F12" s="3"/>
+      <c r="G12" s="2" t="s">
+        <v>79</v>
+      </c>
+      <c r="H12" s="3" t="s">
+        <v>91</v>
+      </c>
+      <c r="I12" s="2" t="s">
+        <v>79</v>
+      </c>
+      <c r="J12" s="2" t="s">
+        <v>78</v>
+      </c>
+      <c r="K12" s="77" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="13" spans="1:11" ht="15" thickBot="1">
+      <c r="B13" s="2" t="s">
+        <v>81</v>
+      </c>
+      <c r="C13" s="3" t="s">
+        <v>124</v>
+      </c>
+      <c r="D13" s="3" t="s">
+        <v>104</v>
+      </c>
+      <c r="E13" s="3" t="s">
+        <v>119</v>
+      </c>
+      <c r="F13" s="3"/>
+      <c r="G13" s="2" t="s">
+        <v>79</v>
+      </c>
+      <c r="H13" s="3" t="s">
+        <v>91</v>
+      </c>
+      <c r="I13" s="2" t="s">
+        <v>79</v>
+      </c>
+      <c r="J13" s="2" t="s">
+        <v>78</v>
+      </c>
+      <c r="K13" s="77" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="14" spans="1:11" ht="15" thickBot="1">
+      <c r="B14" s="2" t="s">
+        <v>81</v>
+      </c>
+      <c r="C14" s="3" t="s">
+        <v>124</v>
+      </c>
+      <c r="D14" s="3" t="s">
+        <v>105</v>
+      </c>
+      <c r="E14" s="3" t="s">
         <v>120</v>
       </c>
-      <c r="D10" s="3" t="s">
-        <v>109</v>
-      </c>
-      <c r="E10" s="3" t="s">
-        <v>101</v>
-      </c>
-      <c r="F10" s="32">
-        <v>15</v>
-      </c>
-      <c r="G10" s="2" t="s">
-        <v>73</v>
-      </c>
-      <c r="H10" s="3" t="s">
-        <v>110</v>
-      </c>
-      <c r="I10" s="32" t="s">
+      <c r="F14" s="3"/>
+      <c r="G14" s="2" t="s">
         <v>79</v>
       </c>
-      <c r="J10" s="6" t="s">
+      <c r="H14" s="3" t="s">
+        <v>80</v>
+      </c>
+      <c r="I14" s="2" t="s">
+        <v>79</v>
+      </c>
+      <c r="J14" s="2" t="s">
         <v>78</v>
       </c>
-      <c r="K10" s="24"/>
+      <c r="K14" s="77" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="15" spans="1:11" ht="15" thickBot="1">
+      <c r="B15" s="2" t="s">
+        <v>81</v>
+      </c>
+      <c r="C15" s="3" t="s">
+        <v>124</v>
+      </c>
+      <c r="D15" s="3" t="s">
+        <v>106</v>
+      </c>
+      <c r="E15" s="3" t="s">
+        <v>121</v>
+      </c>
+      <c r="F15" s="3"/>
+      <c r="G15" s="2" t="s">
+        <v>79</v>
+      </c>
+      <c r="H15" s="3" t="s">
+        <v>80</v>
+      </c>
+      <c r="I15" s="2" t="s">
+        <v>79</v>
+      </c>
+      <c r="J15" s="2" t="s">
+        <v>78</v>
+      </c>
+      <c r="K15" s="77" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="16" spans="1:11">
+      <c r="B16" s="2" t="s">
+        <v>81</v>
+      </c>
+      <c r="C16" s="3" t="s">
+        <v>124</v>
+      </c>
+      <c r="D16" s="3" t="s">
+        <v>107</v>
+      </c>
+      <c r="E16" s="3" t="s">
+        <v>122</v>
+      </c>
+      <c r="F16" s="3">
+        <v>3</v>
+      </c>
+      <c r="G16" s="2" t="s">
+        <v>79</v>
+      </c>
+      <c r="H16" s="3" t="s">
+        <v>80</v>
+      </c>
+      <c r="I16" s="2" t="s">
+        <v>79</v>
+      </c>
+      <c r="J16" s="2" t="s">
+        <v>78</v>
+      </c>
+      <c r="K16" s="77" t="s">
+        <v>39</v>
+      </c>
     </row>
   </sheetData>
   <autoFilter ref="B2:K10" xr:uid="{C02094D6-A0E8-4092-9184-0D999F8AEBED}"/>
@@ -3112,25 +3354,25 @@
           <x14:formula1>
             <xm:f>LISTAS!$C$2:$C$3</xm:f>
           </x14:formula1>
-          <xm:sqref>G3:G10 I3:I1048576</xm:sqref>
+          <xm:sqref>I3:I1048576 G3:G16</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{92736211-7DF3-471C-9486-D14DE458463B}">
           <x14:formula1>
             <xm:f>LISTAS!$B$2:$B$4</xm:f>
           </x14:formula1>
-          <xm:sqref>K3:K10</xm:sqref>
+          <xm:sqref>K3:K16</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{2090DCA7-AC7A-499A-9F11-E7C4B8B63960}">
           <x14:formula1>
             <xm:f>LISTAS!$E$2:$E$5</xm:f>
           </x14:formula1>
-          <xm:sqref>B3:B10 B11:C1048576</xm:sqref>
+          <xm:sqref>C17:C1048576 B3:B1048576</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{E426EE10-F69A-4534-9112-A3EDBE0824B1}">
           <x14:formula1>
             <xm:f>LISTAS!$A$2:$A$5</xm:f>
           </x14:formula1>
-          <xm:sqref>J11:K1048576 J3:J10</xm:sqref>
+          <xm:sqref>J3:J1048576 K17:K1048576</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{A24D8D82-53D3-4AD6-B4DE-A2D4E72177D4}">
           <x14:formula1>
@@ -3281,17 +3523,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="58aa7ded-14a9-4db3-bd1f-b7ef7ff1250a">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="e8557122-6e99-4293-8e44-1c6fc89346af" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Documento" ma:contentTypeID="0x01010025BB7E02133B6442BB1AE44332102476" ma:contentTypeVersion="14" ma:contentTypeDescription="Crear nuevo documento." ma:contentTypeScope="" ma:versionID="a595e19c4197dc6890bbeee52af7f5f1">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="58aa7ded-14a9-4db3-bd1f-b7ef7ff1250a" xmlns:ns3="e8557122-6e99-4293-8e44-1c6fc89346af" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="0001ccacebcf6ea857bfe3329c1c7315" ns2:_="" ns3:_="">
     <xsd:import namespace="58aa7ded-14a9-4db3-bd1f-b7ef7ff1250a"/>
@@ -3520,7 +3751,7 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <?mso-contentType ?>
 <FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
   <Display>DocumentLibraryForm</Display>
@@ -3529,18 +3760,18 @@
 </FormTemplates>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{8754F056-A264-4DA4-8203-DAB0A6DDE008}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="58aa7ded-14a9-4db3-bd1f-b7ef7ff1250a"/>
-    <ds:schemaRef ds:uri="e8557122-6e99-4293-8e44-1c6fc89346af"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="58aa7ded-14a9-4db3-bd1f-b7ef7ff1250a">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="e8557122-6e99-4293-8e44-1c6fc89346af" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{1D3D7F56-302B-465D-923E-40563307D4F1}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -3559,10 +3790,21 @@
 </ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{AEF79A9D-5FC7-4D07-8265-80D988D1A23F}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{8754F056-A264-4DA4-8203-DAB0A6DDE008}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="58aa7ded-14a9-4db3-bd1f-b7ef7ff1250a"/>
+    <ds:schemaRef ds:uri="e8557122-6e99-4293-8e44-1c6fc89346af"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>

</xml_diff>